<commit_message>
feat(template): add required/optional hint row to parent import template
範本第 2 列加入必填/選填/必填之一說明，parser 改為跳過前兩列。

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/assets/templates/parent-import-template.xlsx
+++ b/apps/web/public/assets/templates/parent-import-template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -431,36 +431,65 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>必填</v>
+      </c>
+      <c r="B2" t="str">
+        <v>必填（與Email二擇一）</v>
+      </c>
+      <c r="C2" t="str">
+        <v>必填（與電話二擇一）</v>
+      </c>
+      <c r="D2" t="str">
+        <v>選填</v>
+      </c>
+      <c r="E2" t="str">
+        <v>必填</v>
+      </c>
+      <c r="F2" t="str">
+        <v>必填（見說明頁）</v>
+      </c>
+      <c r="G2" t="str">
+        <v>必填</v>
+      </c>
+      <c r="H2" t="str">
+        <v>選填（YYYY-MM-DD）</v>
+      </c>
+      <c r="I2" t="str">
+        <v>選填（見說明頁）</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
         <v>王美華</v>
       </c>
-      <c r="B2" t="str">
+      <c r="B3" t="str">
         <v>0912345678</v>
       </c>
-      <c r="C2" t="str">
+      <c r="C3" t="str">
+        <v>wang@example.com</v>
+      </c>
+      <c r="D3" t="str">
         <v/>
       </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
+      <c r="E3" t="str">
         <v>王小明</v>
       </c>
-      <c r="F2" t="str">
+      <c r="F3" t="str">
         <v>國一</v>
       </c>
-      <c r="G2" t="str">
+      <c r="G3" t="str">
         <v>台北市立中正國中</v>
       </c>
-      <c r="H2" t="str">
+      <c r="H3" t="str">
         <v>2012-03-15</v>
       </c>
-      <c r="I2" t="str">
+      <c r="I3" t="str">
         <v>男</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(template): set column widths for parent import template
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/assets/templates/parent-import-template.xlsx
+++ b/apps/web/public/assets/templates/parent-import-template.xlsx
@@ -399,6 +399,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I3"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>